<commit_message>
\end{lstfragment} moet aan het begin van de regel staan omdat er anders teveel witruimte verschijnt in TexLive 2020.
</commit_message>
<xml_diff>
--- a/Tabel2020/OmrekenenVerhoudingenKolomXtabu2tabularx.xlsx
+++ b/Tabel2020/OmrekenenVerhoudingenKolomXtabu2tabularx.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BroJZ_git\HR_ELEKTRO\latex-stijl\Tabel2020\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D42A3D0-A95F-4DC8-89D7-D1631ABCA88E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{1CE82A20-8762-40FB-A802-11674BABD60E}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="30930" windowHeight="16890"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -56,7 +55,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -120,18 +122,21 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="2" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Goed" xfId="1" builtinId="26"/>
@@ -447,103 +452,112 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D96A0E3-A3DA-47D3-87ED-EC1DF14E1B14}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="5" t="s">
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="1">
+      <c r="E3" s="1">
         <v>7</v>
-      </c>
-      <c r="D3" s="1">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0</v>
       </c>
       <c r="F3" s="1">
         <v>0</v>
       </c>
-      <c r="G3" s="2">
-        <f>SUM(B3:F3)</f>
-        <v>9</v>
+      <c r="G3" s="1">
+        <v>0</v>
       </c>
       <c r="H3" s="2">
+        <f>SUM(B3:G3)</f>
+        <v>15</v>
+      </c>
+      <c r="I3" s="2">
         <f>COUNTIF(B3:F3,"&lt;&gt;0")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6">
-        <f>B3/$G3*$H3</f>
-        <v>0.44444444444444442</v>
-      </c>
-      <c r="C4" s="6">
-        <f t="shared" ref="C4:F4" si="0">C3/$G3*$H3</f>
-        <v>1.5555555555555556</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="B4" s="7">
+        <f>B3/$H3*$I3</f>
+        <v>0.8</v>
+      </c>
+      <c r="C4" s="7">
+        <f t="shared" ref="C4:G4" si="0">C3/$H3*$I3</f>
+        <v>0.8</v>
+      </c>
+      <c r="D4" s="7">
+        <f t="shared" si="0"/>
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="E4" s="7">
+        <f t="shared" si="0"/>
+        <v>1.8666666666666667</v>
+      </c>
+      <c r="F4" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="E4" s="6">
+      <c r="G4" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F4" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G4" s="2">
-        <f>SUM(B4:F4)</f>
-        <v>2</v>
-      </c>
-      <c r="H4" s="2">
+      <c r="H4" s="7">
+        <f>SUM(B4:G4)</f>
+        <v>4</v>
+      </c>
+      <c r="I4" s="2">
         <f>COUNTIF(B4:F4,"&lt;&gt;0")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>